<commit_message>
:pencil2: Retomando cronograma y roles del equipo
</commit_message>
<xml_diff>
--- a/MATRIZ_RESPONSABILIDADES/planeacion.xlsx
+++ b/MATRIZ_RESPONSABILIDADES/planeacion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduuaa-my.sharepoint.com/personal/al281026_edu_uaa_mx/Documents/Uni/S8/2_ADMIN_SOFT_PROYECTOS/PF/BITACORA/MATRIZ_RESPONSABILIDADES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="62" documentId="13_ncr:1_{604EF1CF-027E-4C19-9D0F-2E4D200D5EFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B79E9FA7-0947-4B13-A506-6CF8A002E0A8}"/>
+  <xr:revisionPtr revIDLastSave="66" documentId="13_ncr:1_{604EF1CF-027E-4C19-9D0F-2E4D200D5EFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{22476CC1-BCFC-4FF0-9EC8-CC8B29939F45}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Grantt" sheetId="1" r:id="rId1"/>
@@ -557,15 +557,15 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -883,7 +883,7 @@
         <v>22</v>
       </c>
       <c r="B1" s="6">
-        <v>46174</v>
+        <v>46148</v>
       </c>
       <c r="D1" s="15" t="s">
         <v>100</v>
@@ -904,35 +904,35 @@
       </c>
       <c r="B3" s="7">
         <f>B1</f>
-        <v>46174</v>
+        <v>46148</v>
       </c>
       <c r="C3" s="7">
         <f>B1+7</f>
-        <v>46181</v>
+        <v>46155</v>
       </c>
       <c r="D3" s="7">
         <f>B1+14</f>
-        <v>46188</v>
+        <v>46162</v>
       </c>
       <c r="E3" s="7">
         <f>B1+21</f>
-        <v>46195</v>
+        <v>46169</v>
       </c>
       <c r="F3" s="7">
         <f>B1+28</f>
-        <v>46202</v>
+        <v>46176</v>
       </c>
       <c r="G3" s="7">
         <f>B1+35</f>
-        <v>46209</v>
+        <v>46183</v>
       </c>
       <c r="H3" s="7">
         <f>B1+42</f>
-        <v>46216</v>
+        <v>46190</v>
       </c>
       <c r="I3" s="7">
         <f>B1+49</f>
-        <v>46223</v>
+        <v>46197</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -1227,16 +1227,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="18"/>
+      <c r="B1" s="20"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="17" t="s">
         <v>84</v>
       </c>
     </row>
@@ -1290,7 +1290,7 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="20">
+      <c r="A9" s="18">
         <v>1.1000000000000001</v>
       </c>
       <c r="B9" s="16" t="s">
@@ -1307,7 +1307,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="18" t="s">
         <v>30</v>
       </c>
       <c r="B10" s="16" t="s">
@@ -1324,7 +1324,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="20" t="s">
+      <c r="A11" s="18" t="s">
         <v>33</v>
       </c>
       <c r="B11" s="16" t="s">
@@ -1341,7 +1341,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="20" t="s">
+      <c r="A12" s="18" t="s">
         <v>35</v>
       </c>
       <c r="B12" s="16" t="s">
@@ -1358,7 +1358,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="20" t="s">
+      <c r="A13" s="18" t="s">
         <v>37</v>
       </c>
       <c r="B13" s="16" t="s">
@@ -1375,7 +1375,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="20" t="s">
+      <c r="A14" s="18" t="s">
         <v>39</v>
       </c>
       <c r="B14" s="16" t="s">
@@ -1392,7 +1392,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="20" t="s">
+      <c r="A15" s="18" t="s">
         <v>42</v>
       </c>
       <c r="B15" s="16" t="s">
@@ -1409,7 +1409,7 @@
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="20" t="s">
+      <c r="A16" s="18" t="s">
         <v>44</v>
       </c>
       <c r="B16" s="16" t="s">
@@ -1426,7 +1426,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="20" t="s">
+      <c r="A17" s="18" t="s">
         <v>46</v>
       </c>
       <c r="B17" s="16" t="s">
@@ -1443,7 +1443,7 @@
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="20" t="s">
+      <c r="A18" s="18" t="s">
         <v>47</v>
       </c>
       <c r="B18" s="16" t="s">
@@ -1460,7 +1460,7 @@
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="20" t="s">
+      <c r="A19" s="18" t="s">
         <v>48</v>
       </c>
       <c r="B19" s="16" t="s">
@@ -1477,7 +1477,7 @@
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="20" t="s">
+      <c r="A20" s="18" t="s">
         <v>50</v>
       </c>
       <c r="B20" s="16" t="s">
@@ -1494,7 +1494,7 @@
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="20" t="s">
+      <c r="A21" s="18" t="s">
         <v>52</v>
       </c>
       <c r="B21" s="16" t="s">
@@ -1511,7 +1511,7 @@
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" s="20" t="s">
+      <c r="A22" s="18" t="s">
         <v>54</v>
       </c>
       <c r="B22" s="16" t="s">
@@ -1528,7 +1528,7 @@
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="20" t="s">
+      <c r="A23" s="18" t="s">
         <v>55</v>
       </c>
       <c r="B23" s="16" t="s">
@@ -1545,7 +1545,7 @@
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" s="20" t="s">
+      <c r="A24" s="18" t="s">
         <v>56</v>
       </c>
       <c r="B24" s="16" t="s">
@@ -1562,7 +1562,7 @@
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" s="20" t="s">
+      <c r="A25" s="18" t="s">
         <v>58</v>
       </c>
       <c r="B25" s="16" t="s">
@@ -1579,7 +1579,7 @@
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A26" s="20" t="s">
+      <c r="A26" s="18" t="s">
         <v>59</v>
       </c>
       <c r="B26" s="16" t="s">
@@ -1596,7 +1596,7 @@
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A27" s="20" t="s">
+      <c r="A27" s="18" t="s">
         <v>61</v>
       </c>
       <c r="B27" s="16" t="s">
@@ -1613,7 +1613,7 @@
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A28" s="20" t="s">
+      <c r="A28" s="18" t="s">
         <v>62</v>
       </c>
       <c r="B28" s="16" t="s">
@@ -1630,7 +1630,7 @@
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A29" s="20" t="s">
+      <c r="A29" s="18" t="s">
         <v>64</v>
       </c>
       <c r="B29" s="16" t="s">
@@ -1647,7 +1647,7 @@
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A30" s="20" t="s">
+      <c r="A30" s="18" t="s">
         <v>66</v>
       </c>
       <c r="B30" s="16" t="s">
@@ -1664,7 +1664,7 @@
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A31" s="20" t="s">
+      <c r="A31" s="18" t="s">
         <v>68</v>
       </c>
       <c r="B31" s="16" t="s">
@@ -1681,7 +1681,7 @@
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A32" s="20" t="s">
+      <c r="A32" s="18" t="s">
         <v>70</v>
       </c>
       <c r="B32" s="16" t="s">
@@ -1698,7 +1698,7 @@
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A33" s="20" t="s">
+      <c r="A33" s="18" t="s">
         <v>72</v>
       </c>
       <c r="B33" s="16" t="s">
@@ -1715,7 +1715,7 @@
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A34" s="20" t="s">
+      <c r="A34" s="18" t="s">
         <v>74</v>
       </c>
       <c r="B34" s="16" t="s">
@@ -1732,7 +1732,7 @@
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A35" s="20">
+      <c r="A35" s="18">
         <v>1.1000000000000001</v>
       </c>
       <c r="B35" s="16" t="s">
@@ -1749,7 +1749,7 @@
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A36" s="20">
+      <c r="A36" s="18">
         <v>1.1100000000000001</v>
       </c>
       <c r="B36" s="16" t="s">
@@ -1766,7 +1766,7 @@
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A37" s="20">
+      <c r="A37" s="18">
         <v>1.1200000000000001</v>
       </c>
       <c r="B37" s="16" t="s">
@@ -1783,7 +1783,7 @@
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A38" s="20" t="s">
+      <c r="A38" s="18" t="s">
         <v>77</v>
       </c>
       <c r="B38" s="16" t="s">
@@ -1800,7 +1800,7 @@
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A39" s="20" t="s">
+      <c r="A39" s="18" t="s">
         <v>79</v>
       </c>
       <c r="B39" s="16" t="s">
@@ -1817,7 +1817,7 @@
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A40" s="20" t="s">
+      <c r="A40" s="18" t="s">
         <v>81</v>
       </c>
       <c r="B40" s="16" t="s">
@@ -1834,7 +1834,7 @@
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A41" s="20">
+      <c r="A41" s="18">
         <v>1.1399999999999999</v>
       </c>
       <c r="B41" s="16" t="s">

</xml_diff>